<commit_message>
Fixed broken Lesson 8 Summary page
I also reordered the summaries to be printed by default and the lesson outcomes to be hidden by default. Opposite the way it was before.
</commit_message>
<xml_diff>
--- a/docs/Data/ClassSurvey.xlsx
+++ b/docs/Data/ClassSurvey.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10208"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ghsaund/Documents/GitHub/BYUI_M221_Book/Data/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C757D82-246B-4D4F-989D-BC3717A67C79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="120" yWindow="225" windowWidth="11475" windowHeight="4785"/>
+    <workbookView xWindow="120" yWindow="800" windowWidth="28740" windowHeight="15740" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -16,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1657" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1694" uniqueCount="90">
   <si>
     <t>F</t>
   </si>
@@ -230,11 +236,68 @@
   <si>
     <t>Heart</t>
   </si>
+  <si>
+    <t>Data collected from a selection of students taking introductory statistics prior to 2020 at BYU-Idaho.</t>
+  </si>
+  <si>
+    <t> The time of day the student was enrolled in Math 221.</t>
+  </si>
+  <si>
+    <t> The gender of the student.</t>
+  </si>
+  <si>
+    <t> The dominant hand of the student.</t>
+  </si>
+  <si>
+    <t> Whether or not the student can "roll their tongue."</t>
+  </si>
+  <si>
+    <t> Whether or not the student can "flip their tongue."</t>
+  </si>
+  <si>
+    <t> Whether or not the student can touch their nose with their tongue.</t>
+  </si>
+  <si>
+    <t> Student's opinion on whether or not the penny should still be in circulation.</t>
+  </si>
+  <si>
+    <t> The class rank of the student: freshman (FR), sophomore (SO), junior (JR), senior (SR).</t>
+  </si>
+  <si>
+    <t> The number of college credits the student had already completed prior to enrolling in Math 221.</t>
+  </si>
+  <si>
+    <t> The heigh of the student in inches.</t>
+  </si>
+  <si>
+    <t> Fear of Statistics 1= Low Fear 7= High Fear</t>
+  </si>
+  <si>
+    <t> Feeling of Math Skils 1=Low Skill 7=High Skill</t>
+  </si>
+  <si>
+    <t> The home state or country of the student.</t>
+  </si>
+  <si>
+    <t> The current or most recent hourly wage the student was earning.</t>
+  </si>
+  <si>
+    <t> The age (in years) the student thought their teacher was at the time of the survey.</t>
+  </si>
+  <si>
+    <t> Whether or not the student went on a date the weekend prior to completing the survey.</t>
+  </si>
+  <si>
+    <t> Students were asked to pick a random number between 1 and 20.</t>
+  </si>
+  <si>
+    <t> The heart rate in beats per minute of the student as they completed the survey.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -276,14 +339,17 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
   </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -321,7 +387,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -393,7 +459,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -566,11 +632,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R184"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:U184"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>53</v>
       </c>
@@ -625,8 +691,11 @@
       <c r="R1" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="2" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>900</v>
       </c>
@@ -681,8 +750,14 @@
       <c r="R2">
         <v>68</v>
       </c>
-    </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T2" t="s">
+        <v>53</v>
+      </c>
+      <c r="U2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="3" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>900</v>
       </c>
@@ -737,8 +812,14 @@
       <c r="R3">
         <v>71</v>
       </c>
-    </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T3" t="s">
+        <v>54</v>
+      </c>
+      <c r="U3" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="4" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>900</v>
       </c>
@@ -793,8 +874,14 @@
       <c r="R4">
         <v>23</v>
       </c>
-    </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T4" t="s">
+        <v>55</v>
+      </c>
+      <c r="U4" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="5" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>900</v>
       </c>
@@ -849,8 +936,14 @@
       <c r="R5">
         <v>78</v>
       </c>
-    </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T5" t="s">
+        <v>56</v>
+      </c>
+      <c r="U5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="6" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>900</v>
       </c>
@@ -905,8 +998,14 @@
       <c r="R6">
         <v>73</v>
       </c>
-    </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T6" t="s">
+        <v>57</v>
+      </c>
+      <c r="U6" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="7" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>900</v>
       </c>
@@ -961,8 +1060,14 @@
       <c r="R7">
         <v>100</v>
       </c>
-    </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T7" t="s">
+        <v>58</v>
+      </c>
+      <c r="U7" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="8" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>900</v>
       </c>
@@ -1017,8 +1122,14 @@
       <c r="R8">
         <v>74</v>
       </c>
-    </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T8" t="s">
+        <v>59</v>
+      </c>
+      <c r="U8" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="9" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>900</v>
       </c>
@@ -1073,8 +1184,14 @@
       <c r="R9">
         <v>62</v>
       </c>
-    </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T9" t="s">
+        <v>60</v>
+      </c>
+      <c r="U9" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="10" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>900</v>
       </c>
@@ -1126,8 +1243,14 @@
       <c r="R10">
         <v>45</v>
       </c>
-    </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T10" t="s">
+        <v>61</v>
+      </c>
+      <c r="U10" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="11" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>900</v>
       </c>
@@ -1179,8 +1302,14 @@
       <c r="R11">
         <v>60</v>
       </c>
-    </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T11" t="s">
+        <v>62</v>
+      </c>
+      <c r="U11" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="12" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>900</v>
       </c>
@@ -1235,8 +1364,14 @@
       <c r="R12">
         <v>62</v>
       </c>
-    </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T12" t="s">
+        <v>63</v>
+      </c>
+      <c r="U12" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="13" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>900</v>
       </c>
@@ -1288,8 +1423,14 @@
       <c r="Q13">
         <v>13</v>
       </c>
-    </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T13" t="s">
+        <v>64</v>
+      </c>
+      <c r="U13" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="14" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>900</v>
       </c>
@@ -1344,8 +1485,14 @@
       <c r="R14">
         <v>93</v>
       </c>
-    </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T14" t="s">
+        <v>65</v>
+      </c>
+      <c r="U14" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="15" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>900</v>
       </c>
@@ -1400,8 +1547,14 @@
       <c r="R15">
         <v>90</v>
       </c>
-    </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T15" t="s">
+        <v>66</v>
+      </c>
+      <c r="U15" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="16" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>900</v>
       </c>
@@ -1453,8 +1606,14 @@
       <c r="Q16">
         <v>7</v>
       </c>
-    </row>
-    <row r="17" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T16" t="s">
+        <v>67</v>
+      </c>
+      <c r="U16" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="17" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>900</v>
       </c>
@@ -1509,8 +1668,14 @@
       <c r="R17">
         <v>78</v>
       </c>
-    </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T17" t="s">
+        <v>68</v>
+      </c>
+      <c r="U17" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="18" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>900</v>
       </c>
@@ -1562,8 +1727,14 @@
       <c r="Q18">
         <v>5</v>
       </c>
-    </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T18" t="s">
+        <v>69</v>
+      </c>
+      <c r="U18" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="19" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>900</v>
       </c>
@@ -1615,8 +1786,14 @@
       <c r="Q19">
         <v>12</v>
       </c>
-    </row>
-    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T19" t="s">
+        <v>70</v>
+      </c>
+      <c r="U19" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="20" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>900</v>
       </c>
@@ -1672,7 +1849,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>900</v>
       </c>
@@ -1728,7 +1905,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>900</v>
       </c>
@@ -1784,7 +1961,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>900</v>
       </c>
@@ -1837,7 +2014,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>900</v>
       </c>
@@ -1893,7 +2070,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>1015</v>
       </c>
@@ -1949,7 +2126,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="26" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>1015</v>
       </c>
@@ -2002,7 +2179,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="27" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>1245</v>
       </c>
@@ -2058,7 +2235,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="28" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>1245</v>
       </c>
@@ -2114,7 +2291,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="29" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>1245</v>
       </c>
@@ -2170,7 +2347,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="30" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>1245</v>
       </c>
@@ -2226,7 +2403,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="31" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>1245</v>
       </c>
@@ -2282,7 +2459,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="32" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>1245</v>
       </c>
@@ -2338,7 +2515,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="33" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>1245</v>
       </c>
@@ -2394,7 +2571,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="34" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>1245</v>
       </c>
@@ -2450,7 +2627,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="35" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>1245</v>
       </c>
@@ -2506,7 +2683,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="36" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>1245</v>
       </c>
@@ -2562,7 +2739,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="37" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>1245</v>
       </c>
@@ -2618,7 +2795,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="38" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>1245</v>
       </c>
@@ -2674,7 +2851,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="39" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>1245</v>
       </c>
@@ -2730,7 +2907,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="40" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>1245</v>
       </c>
@@ -2786,7 +2963,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="41" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>1245</v>
       </c>
@@ -2842,7 +3019,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="42" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>1245</v>
       </c>
@@ -2898,7 +3075,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="43" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>1245</v>
       </c>
@@ -2954,7 +3131,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="44" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>1245</v>
       </c>
@@ -3010,7 +3187,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="45" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A45">
         <v>1245</v>
       </c>
@@ -3066,7 +3243,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="46" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A46">
         <v>1245</v>
       </c>
@@ -3119,7 +3296,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="47" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>1245</v>
       </c>
@@ -3172,7 +3349,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="48" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>1245</v>
       </c>
@@ -3228,7 +3405,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="49" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>1245</v>
       </c>
@@ -3284,7 +3461,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="50" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A50">
         <v>1245</v>
       </c>
@@ -3340,7 +3517,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="51" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A51">
         <v>1245</v>
       </c>
@@ -3396,7 +3573,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="52" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A52">
         <v>1245</v>
       </c>
@@ -3449,7 +3626,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="53" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A53">
         <v>1245</v>
       </c>
@@ -3505,7 +3682,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="54" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A54">
         <v>1245</v>
       </c>
@@ -3561,7 +3738,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="55" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A55">
         <v>1245</v>
       </c>
@@ -3617,7 +3794,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="56" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A56">
         <v>315</v>
       </c>
@@ -3673,7 +3850,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="57" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A57">
         <v>315</v>
       </c>
@@ -3726,7 +3903,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="58" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A58">
         <v>315</v>
       </c>
@@ -3776,7 +3953,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="59" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A59">
         <v>315</v>
       </c>
@@ -3829,7 +4006,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="60" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A60">
         <v>315</v>
       </c>
@@ -3885,7 +4062,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="61" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A61">
         <v>315</v>
       </c>
@@ -3938,7 +4115,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="62" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A62">
         <v>315</v>
       </c>
@@ -3991,7 +4168,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="63" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A63">
         <v>315</v>
       </c>
@@ -4044,7 +4221,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="64" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A64">
         <v>315</v>
       </c>
@@ -4094,7 +4271,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="65" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A65">
         <v>315</v>
       </c>
@@ -4150,7 +4327,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="66" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A66">
         <v>315</v>
       </c>
@@ -4203,7 +4380,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="67" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A67">
         <v>315</v>
       </c>
@@ -4259,7 +4436,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="68" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A68">
         <v>315</v>
       </c>
@@ -4315,7 +4492,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="69" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A69">
         <v>315</v>
       </c>
@@ -4371,7 +4548,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="70" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A70">
         <v>315</v>
       </c>
@@ -4427,7 +4604,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="71" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A71">
         <v>315</v>
       </c>
@@ -4483,7 +4660,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="72" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A72">
         <v>315</v>
       </c>
@@ -4539,7 +4716,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="73" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A73">
         <v>315</v>
       </c>
@@ -4595,7 +4772,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="74" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A74">
         <v>315</v>
       </c>
@@ -4651,7 +4828,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="75" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A75">
         <v>315</v>
       </c>
@@ -4704,7 +4881,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="76" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A76">
         <v>315</v>
       </c>
@@ -4760,7 +4937,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="77" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A77">
         <v>315</v>
       </c>
@@ -4816,7 +4993,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="78" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A78">
         <v>315</v>
       </c>
@@ -4869,7 +5046,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="79" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A79">
         <v>315</v>
       </c>
@@ -4922,7 +5099,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="80" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A80">
         <v>315</v>
       </c>
@@ -4978,7 +5155,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="81" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A81">
         <v>500</v>
       </c>
@@ -5034,7 +5211,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="82" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A82">
         <v>500</v>
       </c>
@@ -5090,7 +5267,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="83" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A83">
         <v>500</v>
       </c>
@@ -5140,7 +5317,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="84" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A84">
         <v>500</v>
       </c>
@@ -5196,7 +5373,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="85" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A85">
         <v>500</v>
       </c>
@@ -5249,7 +5426,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="86" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A86">
         <v>500</v>
       </c>
@@ -5305,7 +5482,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="87" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A87">
         <v>500</v>
       </c>
@@ -5355,7 +5532,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="88" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A88">
         <v>500</v>
       </c>
@@ -5411,7 +5588,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="89" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A89">
         <v>500</v>
       </c>
@@ -5467,7 +5644,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="90" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A90">
         <v>500</v>
       </c>
@@ -5523,7 +5700,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="91" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A91">
         <v>500</v>
       </c>
@@ -5576,7 +5753,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="92" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A92">
         <v>500</v>
       </c>
@@ -5632,7 +5809,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="93" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A93">
         <v>500</v>
       </c>
@@ -5688,7 +5865,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="94" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A94">
         <v>500</v>
       </c>
@@ -5744,7 +5921,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="95" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A95">
         <v>500</v>
       </c>
@@ -5800,7 +5977,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="96" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A96">
         <v>500</v>
       </c>
@@ -5856,7 +6033,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="97" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A97">
         <v>900</v>
       </c>
@@ -5912,7 +6089,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="98" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A98">
         <v>900</v>
       </c>
@@ -5968,7 +6145,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="99" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A99">
         <v>900</v>
       </c>
@@ -6024,7 +6201,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="100" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A100">
         <v>900</v>
       </c>
@@ -6080,7 +6257,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="101" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A101">
         <v>900</v>
       </c>
@@ -6136,7 +6313,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="102" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A102">
         <v>900</v>
       </c>
@@ -6192,7 +6369,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="103" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A103">
         <v>900</v>
       </c>
@@ -6248,7 +6425,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="104" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A104">
         <v>900</v>
       </c>
@@ -6304,7 +6481,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="105" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A105">
         <v>900</v>
       </c>
@@ -6360,7 +6537,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="106" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A106">
         <v>900</v>
       </c>
@@ -6413,7 +6590,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="107" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A107">
         <v>900</v>
       </c>
@@ -6469,7 +6646,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="108" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A108">
         <v>900</v>
       </c>
@@ -6525,7 +6702,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="109" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A109">
         <v>900</v>
       </c>
@@ -6581,7 +6758,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="110" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A110">
         <v>900</v>
       </c>
@@ -6637,7 +6814,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="111" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A111">
         <v>900</v>
       </c>
@@ -6690,7 +6867,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="112" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A112">
         <v>900</v>
       </c>
@@ -6746,7 +6923,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="113" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A113">
         <v>900</v>
       </c>
@@ -6802,7 +6979,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="114" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A114">
         <v>900</v>
       </c>
@@ -6858,7 +7035,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="115" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A115">
         <v>900</v>
       </c>
@@ -6908,7 +7085,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="116" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A116">
         <v>900</v>
       </c>
@@ -6964,7 +7141,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="117" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A117">
         <v>900</v>
       </c>
@@ -7020,7 +7197,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="118" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A118">
         <v>900</v>
       </c>
@@ -7076,7 +7253,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="119" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A119">
         <v>900</v>
       </c>
@@ -7126,7 +7303,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="120" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A120">
         <v>900</v>
       </c>
@@ -7182,7 +7359,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="121" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A121">
         <v>1015</v>
       </c>
@@ -7238,7 +7415,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="122" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A122">
         <v>1015</v>
       </c>
@@ -7294,7 +7471,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="123" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A123">
         <v>1015</v>
       </c>
@@ -7350,7 +7527,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="124" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A124">
         <v>1015</v>
       </c>
@@ -7406,7 +7583,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="125" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A125">
         <v>1015</v>
       </c>
@@ -7462,7 +7639,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="126" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A126">
         <v>1015</v>
       </c>
@@ -7518,7 +7695,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="127" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A127">
         <v>1245</v>
       </c>
@@ -7571,7 +7748,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="128" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A128">
         <v>1245</v>
       </c>
@@ -7627,7 +7804,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="129" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A129">
         <v>1245</v>
       </c>
@@ -7683,7 +7860,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="130" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A130">
         <v>1245</v>
       </c>
@@ -7739,7 +7916,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="131" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A131">
         <v>1245</v>
       </c>
@@ -7795,7 +7972,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="132" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A132">
         <v>1245</v>
       </c>
@@ -7851,7 +8028,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="133" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A133">
         <v>1245</v>
       </c>
@@ -7907,7 +8084,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="134" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A134">
         <v>1245</v>
       </c>
@@ -7963,7 +8140,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="135" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A135">
         <v>1245</v>
       </c>
@@ -8019,7 +8196,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="136" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A136">
         <v>1245</v>
       </c>
@@ -8075,7 +8252,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="137" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A137">
         <v>1245</v>
       </c>
@@ -8131,7 +8308,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="138" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A138">
         <v>1245</v>
       </c>
@@ -8187,7 +8364,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="139" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A139">
         <v>1245</v>
       </c>
@@ -8243,7 +8420,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="140" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A140">
         <v>1245</v>
       </c>
@@ -8296,7 +8473,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="141" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A141">
         <v>1245</v>
       </c>
@@ -8352,7 +8529,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="142" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A142">
         <v>1245</v>
       </c>
@@ -8408,7 +8585,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="143" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A143">
         <v>1245</v>
       </c>
@@ -8464,7 +8641,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="144" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A144">
         <v>1245</v>
       </c>
@@ -8517,7 +8694,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="145" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A145">
         <v>1245</v>
       </c>
@@ -8573,7 +8750,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="146" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A146">
         <v>1245</v>
       </c>
@@ -8629,7 +8806,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="147" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A147">
         <v>1245</v>
       </c>
@@ -8685,7 +8862,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="148" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A148">
         <v>1245</v>
       </c>
@@ -8741,7 +8918,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="149" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A149">
         <v>315</v>
       </c>
@@ -8797,7 +8974,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="150" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A150">
         <v>315</v>
       </c>
@@ -8853,7 +9030,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="151" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A151">
         <v>315</v>
       </c>
@@ -8906,7 +9083,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="152" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A152">
         <v>315</v>
       </c>
@@ -8962,7 +9139,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="153" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A153">
         <v>315</v>
       </c>
@@ -9018,7 +9195,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="154" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A154">
         <v>315</v>
       </c>
@@ -9071,7 +9248,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="155" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A155">
         <v>315</v>
       </c>
@@ -9124,7 +9301,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="156" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A156">
         <v>315</v>
       </c>
@@ -9177,7 +9354,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="157" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A157">
         <v>315</v>
       </c>
@@ -9233,7 +9410,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="158" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A158">
         <v>315</v>
       </c>
@@ -9289,7 +9466,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="159" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A159">
         <v>315</v>
       </c>
@@ -9345,7 +9522,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="160" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A160">
         <v>315</v>
       </c>
@@ -9401,7 +9578,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="161" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A161">
         <v>315</v>
       </c>
@@ -9454,7 +9631,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="162" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A162">
         <v>315</v>
       </c>
@@ -9510,7 +9687,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="163" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A163">
         <v>315</v>
       </c>
@@ -9566,7 +9743,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="164" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A164">
         <v>315</v>
       </c>
@@ -9622,7 +9799,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="165" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A165">
         <v>315</v>
       </c>
@@ -9678,7 +9855,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="166" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A166">
         <v>315</v>
       </c>
@@ -9734,7 +9911,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="167" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A167">
         <v>315</v>
       </c>
@@ -9790,7 +9967,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="168" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A168">
         <v>315</v>
       </c>
@@ -9846,7 +10023,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="169" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A169">
         <v>315</v>
       </c>
@@ -9902,7 +10079,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="170" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A170">
         <v>500</v>
       </c>
@@ -9958,7 +10135,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="171" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A171">
         <v>500</v>
       </c>
@@ -10014,7 +10191,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="172" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A172">
         <v>500</v>
       </c>
@@ -10070,7 +10247,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="173" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A173">
         <v>500</v>
       </c>
@@ -10123,7 +10300,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="174" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A174">
         <v>500</v>
       </c>
@@ -10179,7 +10356,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="175" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A175">
         <v>500</v>
       </c>
@@ -10235,7 +10412,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="176" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A176">
         <v>500</v>
       </c>
@@ -10291,7 +10468,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="177" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A177">
         <v>500</v>
       </c>
@@ -10347,7 +10524,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="178" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A178">
         <v>500</v>
       </c>
@@ -10403,7 +10580,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="179" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A179">
         <v>500</v>
       </c>
@@ -10459,7 +10636,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="180" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A180">
         <v>500</v>
       </c>
@@ -10515,7 +10692,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="181" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A181">
         <v>500</v>
       </c>
@@ -10571,7 +10748,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="182" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A182">
         <v>500</v>
       </c>
@@ -10624,7 +10801,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="183" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A183">
         <v>500</v>
       </c>
@@ -10680,7 +10857,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="184" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A184">
         <v>500</v>
       </c>
@@ -10737,7 +10914,7 @@
       </c>
     </row>
   </sheetData>
-  <sortState ref="A2:R184">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:R184">
     <sortCondition ref="B2"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -10745,18 +10922,18 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>